<commit_message>
Add UK/DE create feeds (4 templates) and refreshed UK/DE listings
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XTewxUJQKBNDwnYyc7b6kM
</commit_message>
<xml_diff>
--- a/Listings_UK_DE_new_products_2026-10-22.xlsx
+++ b/Listings_UK_DE_new_products_2026-10-22.xlsx
@@ -538,7 +538,7 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Источник ключей</t>
+          <t>Ключи / источник</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Cerebro UK: hair regrowth oil (hair conditioner/shampoo), proxy</t>
+          <t>shampoo 92620; conditioner 30681; hair conditioner 9246</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>Cerebro UK: hair regrowth oil, proxy</t>
+          <t>conditioner 30681; hair conditioner 9246</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>Cerebro UK: hair regrowth oil, proxy</t>
+          <t>shampoo 92620; argan oil 8518</t>
         </is>
       </c>
     </row>
@@ -882,7 +882,7 @@
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>Cerebro UK: hair regrowth oil, proxy</t>
+          <t>conditioner; hair conditioner 9246; argan oil 8518</t>
         </is>
       </c>
     </row>
@@ -902,11 +902,11 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>ZAptieka Natural Face Balm 60 ml with Shea Butter, Myrrh and Frankincense</t>
+          <t>ZAptieka Face Balm 60 ml, Natural Face Moisturiser with Shea Butter, Myrrh</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -968,7 +968,7 @@
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>Cerebro UK: night creme (face cream/moisturiser), proxy</t>
+          <t>face moisturiser 15125; face cream 17488; moisturiser 29973</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>Cerebro UK: night creme (eye cream 23169), proxy</t>
+          <t>eye cream 23169 (Night creme)</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>нет выгрузки Cerebro под категорию — ключи по рынку, объём не подтверждён</t>
+          <t>нет Cerebro под face serum (есть только X-Ray): proxy</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>нет выгрузки Cerebro под категорию — ключи по рынку, объём не подтверждён</t>
+          <t>нет Cerebro под nail oil (только X-Ray): proxy, из прежнего SEO nail oil 6216</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>нет выгрузки Cerebro под категорию — ключи по рынку, объём не подтверждён</t>
+          <t>нет выгрузки Cerebro UK по ресницам</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1438,7 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Источник ключей</t>
+          <t>Ключи / источник</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1524,7 @@
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Cerebro DE: shampoo (shampoo damen/herren)</t>
+          <t>shampoo 19706; shampoo damen 8568; shampoo herren 4684</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>Cerebro DE: shampoo (conditioner 6039)</t>
+          <t>conditioner 5814; haarkur 3960</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>Cerebro DE: shampoo</t>
+          <t>shampoo 19706; shampoo damen 8568</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>Cerebro DE: shampoo (conditioner)</t>
+          <t>conditioner 5814; haarkur 3960</t>
         </is>
       </c>
     </row>
@@ -1802,11 +1802,11 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>ZAptieka Gesichtsbalsam 60 ml mit Sheabutter, Myrrhe und Weihrauch</t>
+          <t>ZAptieka Gesichtscreme 60 ml, Balsam mit Sheabutter, Myrrhe und Weihrauch</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -1868,7 +1868,7 @@
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>Cerebro DE: Gesichtscreme</t>
+          <t>gesichtscreme 10274; gesichtspflege 8554</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>Cerebro DE: Gesichtscreme (augencreme 7978)</t>
+          <t>augencreme 8868</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Einfache Formel: 100 % natürliche Öle, wasserfrei und ohne zugesetzten Duftstoff, reich an natürlichen Fettsäuren und Vitamin E</t>
+          <t>Einfache Formel: 100 % natürliche Öle, ohne Hormone, wasserfrei und ohne zugesetzten Duftstoff, reich an natürlichen Fettsäuren und Vitamin E</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>нет выгрузки Cerebro под категорию — ключи по рынку, объём не подтверждён</t>
+          <t>serum 2876; serum gesicht 2546; hyaluron serum 8960 (не про этот состав)</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>нет выгрузки Cerebro под категорию — ключи по рынку, объём не подтверждён</t>
+          <t>rizinusöl 29128; propolis nagelserum 9976; Nagelpflege: proxy</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>нет выгрузки Cerebro под категорию — ключи по рынку, объём не подтверждён</t>
+          <t>wimpernserum 25042; lash serum 4286; wimpernserum ohne hormone 3032</t>
         </is>
       </c>
     </row>
@@ -2227,65 +2227,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="160" customWidth="1" min="1" max="1"/>
+    <col width="170" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Листинги UK и DE для 9 новых товаров (Ввод в ассортимент). Лимиты: Title 75, Highlight 125, буллет 10-255, Description 2000, backend 249 байт.</t>
+          <t>Лимиты: Title 75, Highlight 125, буллет 10-255, Description 2000, backend 249 байт.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Товары 1-6: тексты из Task - SEO.xlsx. Изменены только кондиционеры (№2, №4): убрано масло ши, его нет в INCI (Title, Bullet 1, первое предложение Description).</t>
+          <t>Товары 1-6: тексты Task - SEO.xlsx; кондиционеры: убрано масло ши (нет в INCI). Заголовки бальзама для лица подогнаны под Cerebro (UK face moisturiser; DE Gesichtscreme).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Товары 7-9 (ресницы, сыворотка лаванда, ногти): тексты новые, строго по INCI и данным ПМ.</t>
+          <t>Товары 7-9: тексты новые по INCI и данным ПМ. Не использованы заявления ПМ про ускорение роста, отбеливание ногтей, противогрибковое, омоложение, отёки/тёмные круги.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Не использованы заявления ПМ: ускорение роста ресниц/ногтей, отбеливание ногтей, противогрибковое действие, омоложение, уменьшение отёков и тёмных кругов, противовоспалительное действие, 'без простагландинов и гормонов'.</t>
+          <t>Cerebro: выгрузки в основном брендовые и не по теме (kerastase, olaplex, cerave, medicube). Бренды не использованы. GB_AMAZON_Eye cream.xlsx по содержанию шампунь/кондиционер, не eye cream. GB: нет Cerebro по ресницам и отдельно по шампуню; Face serum oil и Nail oil только X-Ray.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cerebro/X-Ray в папках DE и UK собраны по другим категориям (крем, шампунь DE; лосьон, ночной крем, мочалки, масла, мыло, hair regrowth UK). Под кондиционер, бальзам для глаз, ресницы, сыворотку для лица и масло для ногтей прямых выгрузок нет: ключи подобраны как proxy, объёмы не подтверждены.</t>
+          <t>DE ресницы: 'ohne Hormone' и 'prostaglandinfrei' взяты из данных ПМ.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Бренды конкурентов из выгрузок (kerastase, olaplex, cerave, medicube и др.) не использованы.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Фото ладана (шампунь/кондиционер): флакон 100 мл с бейджем TRAVEL SIZE, в данных 250 мл. Объём и фото нужно проверить.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Backend у новых товаров: только слова, которых нет в Title/буллетах/Highlight.</t>
+          <t>Фото ладана: флакон 100 мл с бейджем TRAVEL SIZE, в данных 250 мл.</t>
         </is>
       </c>
     </row>

</xml_diff>